<commit_message>
Corrida | SFE-XMOA | 2026-06-17 11:55:25.161473
</commit_message>
<xml_diff>
--- a/indicadores/SFE-XMOA_out.xlsx
+++ b/indicadores/SFE-XMOA_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="441">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Exportaciones de MOA con origen en la provincia de Santa Fe</t>
+    <t xml:space="preserve">Exportaciones de MOA</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -71,6 +71,12 @@
     <t xml:space="preserve">Regresores</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -104,13 +110,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">21/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">fleiva</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1833,9 +1839,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1846,7 +1856,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1860,12 +1870,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.222860157601949</v>
+        <v>0.22258386297064</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1876,7 +1886,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1904,7 +1914,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1918,12 +1928,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.0331762372999909</v>
+        <v>0.0325832032130097</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1946,7 +1956,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -1960,7 +1970,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -1974,7 +1984,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -1988,12 +1998,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.182114900304534</v>
+        <v>0.169560108212235</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2004,7 +2014,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2018,12 +2028,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.666555352740306</v>
+        <v>0.630595443175934</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2166,10 +2176,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2182,10 +2192,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2209,66 +2219,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="P1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="R1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>216.99102159</v>
@@ -2321,7 +2331,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>196.43125606</v>
@@ -2378,7 +2388,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>208.54054545</v>
@@ -2435,7 +2445,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>267.88960044</v>
@@ -2492,7 +2502,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>297.5597505</v>
@@ -2549,7 +2559,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>302.59416211</v>
@@ -2606,7 +2616,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>358.83737623</v>
@@ -2663,7 +2673,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>312.49587736</v>
@@ -2720,7 +2730,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>382.8496836</v>
@@ -2777,7 +2787,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>344.44612777</v>
@@ -2834,7 +2844,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>345.05194875</v>
@@ -2891,7 +2901,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>307.64148919</v>
@@ -2948,7 +2958,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>345.55213628</v>
@@ -3007,7 +3017,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>301.68715726</v>
@@ -3066,7 +3076,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>284.15129423</v>
@@ -3125,7 +3135,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>300.93687869</v>
@@ -3184,7 +3194,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>432.78403706</v>
@@ -3243,7 +3253,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>402.12068136</v>
@@ -3302,7 +3312,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>438.16453258</v>
@@ -3361,7 +3371,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>391.3154945</v>
@@ -3420,7 +3430,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>404.89604032</v>
@@ -3479,7 +3489,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>430.34113463</v>
@@ -3538,7 +3548,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>462.58342535</v>
@@ -3597,7 +3607,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>431.74173692</v>
@@ -3656,7 +3666,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>440.56542063</v>
@@ -3715,7 +3725,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>462.23405526</v>
@@ -3774,7 +3784,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>388.28020741</v>
@@ -3833,7 +3843,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>443.75298477</v>
@@ -3892,7 +3902,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>617.46369267</v>
@@ -3951,7 +3961,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>423.25867187</v>
@@ -4010,7 +4020,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>492.46173423</v>
@@ -4069,7 +4079,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>423.60322852</v>
@@ -4128,7 +4138,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>368.00093789</v>
@@ -4187,7 +4197,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>380.26478433</v>
@@ -4246,7 +4256,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>413.09397617</v>
@@ -4305,7 +4315,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>375.04581976</v>
@@ -4364,7 +4374,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>388.21121886</v>
@@ -4423,7 +4433,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>356.34015848</v>
@@ -4482,7 +4492,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>410.9639342</v>
@@ -4541,7 +4551,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>449.59304481</v>
@@ -4600,7 +4610,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>473.56035204</v>
@@ -4659,7 +4669,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>481.555464</v>
@@ -4718,7 +4728,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>498.113015</v>
@@ -4777,7 +4787,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>553.2325187</v>
@@ -4836,7 +4846,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>484.52856675</v>
@@ -4895,7 +4905,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>483.09553864</v>
@@ -4954,7 +4964,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>444.65145618</v>
@@ -5013,7 +5023,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>488.39821777</v>
@@ -5072,7 +5082,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>492.81771622</v>
@@ -5131,7 +5141,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>448.23722985</v>
@@ -5190,7 +5200,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>471.93286366</v>
@@ -5249,7 +5259,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>490.25168964</v>
@@ -5308,7 +5318,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>606.94632441</v>
@@ -5367,7 +5377,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>499.79302246</v>
@@ -5426,7 +5436,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>578.43456976</v>
@@ -5485,7 +5495,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>569.94909882</v>
@@ -5544,7 +5554,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>564.19389647</v>
@@ -5603,7 +5613,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>659.45846378</v>
@@ -5662,7 +5672,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>595.59770899</v>
@@ -5721,7 +5731,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>681.91288233</v>
@@ -5780,7 +5790,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>488.13569544</v>
@@ -5839,7 +5849,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>624.37529027</v>
@@ -5898,7 +5908,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>570.9495507</v>
@@ -5957,7 +5967,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>612.90478828</v>
@@ -6016,7 +6026,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>787.12579808</v>
@@ -6075,7 +6085,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>718.72533348</v>
@@ -6134,7 +6144,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>798.76033633</v>
@@ -6193,7 +6203,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>777.40045236</v>
@@ -6252,7 +6262,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>800.79670923</v>
@@ -6311,7 +6321,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>1040.14146317</v>
@@ -6370,7 +6380,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>918.03975612</v>
@@ -6429,7 +6439,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>1006.89431755</v>
@@ -6488,7 +6498,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>1017.46728027</v>
@@ -6547,7 +6557,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>839.37313865</v>
@@ -6606,7 +6616,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>592.09892063</v>
@@ -6665,7 +6675,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>821.70002099</v>
@@ -6724,7 +6734,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>1177.07493742</v>
@@ -6783,7 +6793,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>816.74396324</v>
@@ -6842,7 +6852,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>923.51851073</v>
@@ -6901,7 +6911,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>1223.88638482</v>
@@ -6960,7 +6970,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>1158.08989122</v>
@@ -7019,7 +7029,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>964.50254754</v>
@@ -7078,7 +7088,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>692.93381443</v>
@@ -7137,7 +7147,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>673.87465399</v>
@@ -7196,7 +7206,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>721.43945722</v>
@@ -7255,7 +7265,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>732.89729706</v>
@@ -7314,7 +7324,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>690.16246764</v>
@@ -7373,7 +7383,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>948.9435225</v>
@@ -7432,7 +7442,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>993.53079302</v>
@@ -7491,7 +7501,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>1164.34738944</v>
@@ -7550,7 +7560,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>946.604019</v>
@@ -7609,7 +7619,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>751.13947133</v>
@@ -7668,7 +7678,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>757.1539476</v>
@@ -7727,7 +7737,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>784.6050285</v>
@@ -7786,7 +7796,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>793.08336922</v>
@@ -7845,7 +7855,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>729.71757911</v>
@@ -7904,7 +7914,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>581.22189498</v>
@@ -7963,7 +7973,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>587.8708663</v>
@@ -8022,7 +8032,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>427.69308234</v>
@@ -8081,7 +8091,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>937.41907405</v>
@@ -8140,7 +8150,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>1048.0606101</v>
@@ -8199,7 +8209,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>996.43640242</v>
@@ -8258,7 +8268,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>1033.30494223</v>
@@ -8317,7 +8327,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>923.79825899</v>
@@ -8376,7 +8386,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>1057.38303005</v>
@@ -8435,7 +8445,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>1072.00755772</v>
@@ -8494,7 +8504,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>1024.85555939</v>
@@ -8553,7 +8563,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>822.61219451</v>
@@ -8612,7 +8622,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>837.03707781</v>
@@ -8671,7 +8681,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>850.48786158</v>
@@ -8730,7 +8740,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>947.30951544</v>
@@ -8789,7 +8799,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>1098.22620563</v>
@@ -8848,7 +8858,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>1378.80306025</v>
@@ -8907,7 +8917,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>1265.31719595</v>
@@ -8966,7 +8976,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>917.65177806</v>
@@ -9025,7 +9035,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>1236.70790715</v>
@@ -9084,7 +9094,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>1099.17601322</v>
@@ -9143,7 +9153,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>1070.54454325</v>
@@ -9202,7 +9212,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>861.56322768</v>
@@ -9261,7 +9271,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>790.36157194</v>
@@ -9320,7 +9330,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>679.30071736</v>
@@ -9379,7 +9389,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>934.90769228</v>
@@ -9438,7 +9448,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>780.2297478</v>
@@ -9497,7 +9507,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>927.49544523</v>
@@ -9556,7 +9566,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>1284.05328202</v>
@@ -9615,7 +9625,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>1126.26660009</v>
@@ -9674,7 +9684,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>1183.76907772</v>
@@ -9733,7 +9743,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>1273.2002696</v>
@@ -9792,7 +9802,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>1085.92810283</v>
@@ -9851,7 +9861,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>956.31627192</v>
@@ -9910,7 +9920,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>945.81309737</v>
@@ -9969,7 +9979,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>747.0109956</v>
@@ -10028,7 +10038,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>685.06390893</v>
@@ -10087,7 +10097,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>710.5636012</v>
@@ -10146,7 +10156,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>535.815433</v>
@@ -10205,7 +10215,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>1087.80120709</v>
@@ -10264,7 +10274,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>1355.78099778</v>
@@ -10323,7 +10333,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>1168.25053615</v>
@@ -10382,7 +10392,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>1232.68874522</v>
@@ -10441,7 +10451,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>1348.55170561</v>
@@ -10500,7 +10510,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>1037.98363289</v>
@@ -10559,7 +10569,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>789.63532762</v>
@@ -10618,7 +10628,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>711.54492774</v>
@@ -10677,7 +10687,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>853.35223222</v>
@@ -10736,7 +10746,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>658.33774635</v>
@@ -10795,7 +10805,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>679.76704316</v>
@@ -10854,7 +10864,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>605.72049706</v>
@@ -10913,7 +10923,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>1540.88338058</v>
@@ -10972,7 +10982,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>1471.9769044</v>
@@ -11031,7 +11041,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>1481.17958645</v>
@@ -11090,7 +11100,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>1157.61950243</v>
@@ -11149,7 +11159,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>1156.6055899</v>
@@ -11208,7 +11218,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>830.36820049</v>
@@ -11267,7 +11277,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>867.35451148</v>
@@ -11326,7 +11336,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>841.59194669</v>
@@ -11385,7 +11395,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>716.71514258</v>
@@ -11444,7 +11454,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>664.69040343</v>
@@ -11503,7 +11513,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>716.32715345</v>
@@ -11562,7 +11572,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>685.86651401</v>
@@ -11621,7 +11631,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>976.82848095</v>
@@ -11680,7 +11690,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>746.22623185</v>
@@ -11739,7 +11749,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>1110.72845495</v>
@@ -11798,7 +11808,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>1213.43973002</v>
@@ -11857,7 +11867,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>928.72658374</v>
@@ -11916,7 +11926,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>967.27115645</v>
@@ -11975,7 +11985,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>871.86313634</v>
@@ -12034,7 +12044,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>757.40286606</v>
@@ -12093,7 +12103,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>579.28941723</v>
@@ -12152,7 +12162,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>850.37960036</v>
@@ -12211,7 +12221,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>807.98698305</v>
@@ -12270,7 +12280,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>750.14203665</v>
@@ -12329,7 +12339,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>854.89615486</v>
@@ -12388,7 +12398,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>992.13867841</v>
@@ -12447,7 +12457,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>932.16724801</v>
@@ -12506,7 +12516,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>815.2874418</v>
@@ -12565,7 +12575,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>1000.59443833</v>
@@ -12624,7 +12634,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>721.52211936</v>
@@ -12683,7 +12693,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>932.70571002</v>
@@ -12742,7 +12752,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>877.9008213</v>
@@ -12801,7 +12811,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>860.22066931</v>
@@ -12860,7 +12870,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>782.81195026</v>
@@ -12919,7 +12929,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>670.62867114</v>
@@ -12978,7 +12988,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>953.93920114</v>
@@ -13037,7 +13047,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>878.63522886</v>
@@ -13096,7 +13106,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>936.17983998</v>
@@ -13155,7 +13165,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>809.34482053</v>
@@ -13214,7 +13224,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>918.15681265</v>
@@ -13273,7 +13283,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>886.70017597</v>
@@ -13332,7 +13342,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>803.32994976</v>
@@ -13391,7 +13401,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>1005.30544434</v>
@@ -13450,7 +13460,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>700.12403551</v>
@@ -13509,7 +13519,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>577.54179048</v>
@@ -13568,7 +13578,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>667.39474034</v>
@@ -13627,7 +13637,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>688.11784582</v>
@@ -13686,7 +13696,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>905.96993472</v>
@@ -13745,7 +13755,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>892.3420507</v>
@@ -13804,7 +13814,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>1003.90763693</v>
@@ -13863,7 +13873,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>850.00556705</v>
@@ -13922,7 +13932,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>936.95417509</v>
@@ -13981,7 +13991,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>924.11978611</v>
@@ -14040,7 +14050,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>891.74320565</v>
@@ -14099,7 +14109,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>927.90314814</v>
@@ -14158,7 +14168,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>650.34237995</v>
@@ -14217,7 +14227,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>723.1293708</v>
@@ -14276,7 +14286,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>776.67083055</v>
@@ -14335,7 +14345,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>759.30163513</v>
@@ -14394,7 +14404,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>738.12790552</v>
@@ -14453,7 +14463,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>812.85530477</v>
@@ -14512,7 +14522,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>1033.78923056</v>
@@ -14571,7 +14581,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>972.72217982</v>
@@ -14630,7 +14640,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>949.80004454</v>
@@ -14689,7 +14699,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>944.57079335</v>
@@ -14748,7 +14758,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>946.01031539</v>
@@ -14807,7 +14817,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>963.4519917</v>
@@ -14866,7 +14876,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>795.21276167</v>
@@ -14925,7 +14935,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>701.00457564</v>
@@ -14984,7 +14994,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>542.08097744</v>
@@ -15043,7 +15053,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>500.72426226</v>
@@ -15102,7 +15112,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>561.95597817</v>
@@ -15161,7 +15171,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>698.55460844</v>
@@ -15220,7 +15230,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>848.49886381</v>
@@ -15279,7 +15289,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>855.92993356</v>
@@ -15338,7 +15348,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>710.57233304</v>
@@ -15397,7 +15407,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>749.69363474</v>
@@ -15456,7 +15466,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>731.46683025</v>
@@ -15515,7 +15525,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>844.82125799</v>
@@ -15574,7 +15584,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>975.4165396</v>
@@ -15633,7 +15643,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>338.38462774</v>
@@ -15692,7 +15702,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>1089.06204943</v>
@@ -15751,7 +15761,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>1038.17502674</v>
@@ -15810,7 +15820,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>1132.76478831</v>
@@ -15869,7 +15879,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>1334.63866486</v>
@@ -15928,7 +15938,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>1219.03663406</v>
@@ -15987,7 +15997,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>1152.72083421</v>
@@ -16046,7 +16056,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>1037.27098722</v>
@@ -16105,7 +16115,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>980.90953366</v>
@@ -16164,7 +16174,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>1189.14789287</v>
@@ -16223,7 +16233,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>1015.71156384</v>
@@ -16282,7 +16292,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>1068.7544253</v>
@@ -16341,7 +16351,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>871.31717259</v>
@@ -16400,7 +16410,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>659.39296101</v>
@@ -16459,7 +16469,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>867.77374298</v>
@@ -16518,7 +16528,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>1058.94476074</v>
@@ -16577,7 +16587,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>1434.35115161</v>
@@ -16636,7 +16646,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>1535.380443</v>
@@ -16695,7 +16705,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>1542.6660248</v>
@@ -16754,7 +16764,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>1102.4853433</v>
@@ -16813,7 +16823,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>1007.88340052</v>
@@ -16872,7 +16882,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>1026.22873732</v>
@@ -16931,7 +16941,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>1035.72121999</v>
@@ -16990,7 +17000,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>1149.10818422</v>
@@ -17049,7 +17059,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>1022.63790637</v>
@@ -17108,7 +17118,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>756.99307615</v>
@@ -17167,7 +17177,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>709.44749718</v>
@@ -17226,7 +17236,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>671.2082043</v>
@@ -17285,7 +17295,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>902.1920084</v>
@@ -17344,7 +17354,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>1106.20531257</v>
@@ -17403,7 +17413,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>861.76475594</v>
@@ -17462,7 +17472,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>732.01799278</v>
@@ -17521,7 +17531,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>753.72998924</v>
@@ -17580,7 +17590,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>583.34604447</v>
@@ -17639,7 +17649,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>560.24980615</v>
@@ -17698,7 +17708,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>573.02011829</v>
@@ -17757,7 +17767,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>656.53825384</v>
@@ -17816,7 +17826,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>738.71671113</v>
@@ -17875,7 +17885,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>783.26343342</v>
@@ -17934,7 +17944,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>853.0025118</v>
@@ -17993,7 +18003,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>952.99052185</v>
@@ -18052,7 +18062,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>1136.72952685</v>
@@ -18111,7 +18121,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>1082.17251831</v>
@@ -18170,7 +18180,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>1009.61861436</v>
@@ -18229,7 +18239,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>911.48962326</v>
@@ -18288,7 +18298,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>1060.53515996</v>
@@ -18347,7 +18357,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>1071.05079901</v>
@@ -18406,7 +18416,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>1128.29315552</v>
@@ -18465,7 +18475,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>996.31460619</v>
@@ -18524,7 +18534,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>856.9987922</v>
@@ -18583,7 +18593,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>920.5870079</v>
@@ -18642,7 +18652,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>889.69759321</v>
@@ -18701,7 +18711,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>937.41207249</v>
@@ -18760,7 +18770,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>894.04460992</v>
@@ -18819,7 +18829,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>991.19672312</v>
@@ -18878,7 +18888,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>1095.10195027</v>
@@ -18937,7 +18947,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>992.87055759</v>
@@ -18996,7 +19006,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>1172.54460675</v>
@@ -19055,7 +19065,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>1035.51863685</v>
@@ -19114,7 +19124,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>1139.41721571</v>
@@ -19173,7 +19183,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>993.95125813</v>
@@ -19232,7 +19242,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>1033.25331883</v>
@@ -19291,7 +19301,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>811.97503727</v>
@@ -19350,7 +19360,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>1300.05421389</v>
@@ -19409,7 +19419,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>1315.13949301</v>
@@ -19468,7 +19478,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B294" s="2"/>
       <c r="C294" s="3" t="n">
@@ -19501,7 +19511,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B295" s="2"/>
       <c r="C295" s="3" t="n">
@@ -19534,7 +19544,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B296" s="2"/>
       <c r="C296" s="3" t="n">
@@ -19567,7 +19577,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B297" s="2"/>
       <c r="C297" s="3" t="n">
@@ -19600,7 +19610,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B298" s="2"/>
       <c r="C298" s="3" t="n">
@@ -19633,7 +19643,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B299" s="2"/>
       <c r="C299" s="3" t="n">
@@ -19666,7 +19676,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B300" s="2"/>
       <c r="C300" s="3" t="n">
@@ -19699,7 +19709,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B301" s="2"/>
       <c r="C301" s="3" t="n">
@@ -19732,7 +19742,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B302" s="2"/>
       <c r="C302" s="3" t="n">
@@ -19765,7 +19775,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B303" s="2"/>
       <c r="C303" s="3" t="n">
@@ -19798,7 +19808,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B304" s="2"/>
       <c r="C304" s="3" t="n">
@@ -19831,7 +19841,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B305" s="2"/>
       <c r="C305" s="3" t="n">
@@ -19864,7 +19874,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B306" s="2"/>
       <c r="C306" s="3"/>
@@ -19887,7 +19897,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B307" s="2"/>
       <c r="C307" s="3"/>
@@ -19910,7 +19920,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B308" s="2"/>
       <c r="C308" s="3"/>
@@ -19933,7 +19943,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B309" s="2"/>
       <c r="C309" s="3"/>
@@ -19956,7 +19966,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B310" s="2"/>
       <c r="C310" s="3"/>
@@ -19979,7 +19989,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B311" s="2"/>
       <c r="C311" s="3"/>
@@ -20002,7 +20012,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B312" s="2"/>
       <c r="C312" s="3"/>
@@ -20025,7 +20035,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B313" s="2"/>
       <c r="C313" s="3"/>
@@ -20048,7 +20058,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B314" s="2"/>
       <c r="C314" s="3"/>
@@ -20071,7 +20081,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B315" s="2"/>
       <c r="C315" s="3"/>
@@ -20094,7 +20104,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B316" s="2"/>
       <c r="C316" s="3"/>
@@ -20117,7 +20127,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B317" s="2"/>
       <c r="C317" s="3"/>
@@ -20140,7 +20150,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B318" s="2"/>
       <c r="C318" s="3"/>
@@ -20163,7 +20173,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B319" s="2"/>
       <c r="C319" s="3"/>
@@ -20186,7 +20196,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B320" s="2"/>
       <c r="C320" s="3"/>
@@ -20209,7 +20219,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B321" s="2"/>
       <c r="C321" s="3"/>
@@ -20232,7 +20242,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B322" s="2"/>
       <c r="C322" s="3"/>
@@ -20255,7 +20265,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B323" s="2"/>
       <c r="C323" s="3"/>
@@ -20278,7 +20288,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B324" s="2"/>
       <c r="C324" s="3"/>
@@ -20301,7 +20311,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B325" s="2"/>
       <c r="C325" s="3"/>
@@ -20324,7 +20334,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B326" s="2"/>
       <c r="C326" s="3"/>
@@ -20347,7 +20357,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B327" s="2"/>
       <c r="C327" s="3"/>
@@ -20370,7 +20380,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B328" s="2"/>
       <c r="C328" s="3"/>
@@ -20393,7 +20403,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B329" s="2"/>
       <c r="C329" s="3"/>
@@ -20416,7 +20426,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B330" s="2"/>
       <c r="C330" s="3"/>
@@ -20439,7 +20449,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B331" s="2"/>
       <c r="C331" s="3"/>
@@ -20462,7 +20472,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B332" s="2"/>
       <c r="C332" s="3"/>
@@ -20485,7 +20495,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B333" s="2"/>
       <c r="C333" s="3"/>
@@ -20508,7 +20518,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B334" s="2"/>
       <c r="C334" s="3"/>
@@ -20531,7 +20541,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B335" s="2"/>
       <c r="C335" s="3"/>
@@ -20554,7 +20564,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B336" s="2"/>
       <c r="C336" s="3"/>
@@ -20577,7 +20587,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B337" s="2"/>
       <c r="C337" s="3"/>
@@ -20600,7 +20610,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B338" s="2"/>
       <c r="C338" s="3"/>
@@ -20623,7 +20633,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B339" s="2"/>
       <c r="C339" s="3"/>
@@ -20646,7 +20656,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B340" s="2"/>
       <c r="C340" s="3"/>
@@ -20669,7 +20679,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B341" s="2"/>
       <c r="C341" s="3"/>
@@ -20692,7 +20702,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B342" s="2"/>
       <c r="C342" s="3"/>
@@ -20715,7 +20725,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B343" s="2"/>
       <c r="C343" s="3"/>
@@ -20738,7 +20748,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B344" s="2"/>
       <c r="C344" s="3"/>
@@ -20761,7 +20771,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B345" s="2"/>
       <c r="C345" s="3"/>
@@ -20784,7 +20794,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B346" s="2"/>
       <c r="C346" s="3"/>
@@ -20807,7 +20817,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B347" s="2"/>
       <c r="C347" s="3"/>
@@ -20830,7 +20840,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B348" s="2"/>
       <c r="C348" s="3"/>
@@ -20853,7 +20863,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B349" s="2"/>
       <c r="C349" s="3"/>
@@ -20887,97 +20897,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
     </row>
   </sheetData>
@@ -21001,7 +21011,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -21011,160 +21021,160 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.0575205346862459</v>
+        <v>0.0605279873450046</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0325370422995509</v>
+        <v>0.0345047793387983</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0540893698970526</v>
+        <v>0.0547550543349535</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.10951658968884</v>
+        <v>0.109664282808583</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.151077793530215</v>
+        <v>0.151400133730989</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.172035912044033</v>
+        <v>0.171582388093477</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.190009693681605</v>
+        <v>0.189284477021176</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.20514531268037</v>
+        <v>0.205255537041313</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.222860157601949</v>
+        <v>0.22258386297064</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.182143452531214</v>
+        <v>0.180508180460083</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.0642357369071212</v>
+        <v>0.0643829913232454</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>-0.00968391214724539</v>
+        <v>-0.00696711732179472</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.00741206643774369</v>
+        <v>0.0103594802777225</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.0429182650406119</v>
+        <v>0.0445114322105607</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0463643924178809</v>
+        <v>0.0470880073055065</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.0088568673974218</v>
+        <v>0.00863152436765892</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0318583559193329</v>
+        <v>-0.032616600766794</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.0614919022197202</v>
+        <v>-0.0622598463482531</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.102046686585891</v>
+        <v>-0.103361780137007</v>
       </c>
     </row>
     <row r="24">

</xml_diff>